<commit_message>
chore: update passive server
</commit_message>
<xml_diff>
--- a/equipment_sequence/manual.xlsx
+++ b/equipment_sequence/manual.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="27945" windowHeight="12375" tabRatio="485" firstSheet="1" activeTab="7"/>
+    <workbookView windowWidth="27945" windowHeight="12375" tabRatio="485" firstSheet="1" activeTab="4"/>
   </bookViews>
   <sheets>
     <sheet name="secs指令" sheetId="14" r:id="rId1"/>
@@ -308,7 +308,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="653" uniqueCount="423">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="657" uniqueCount="426">
   <si>
     <t>direction</t>
   </si>
@@ -1090,6 +1090,15 @@
   </si>
   <si>
     <t>Host 服务监控设备端的服务ip和端口列表</t>
+  </si>
+  <si>
+    <t>equipment_type</t>
+  </si>
+  <si>
+    <t>plc</t>
+  </si>
+  <si>
+    <t>控制设备运行的类型, plc: plc 控制运动, socket:板卡控制运动(通过 socket 和 mes 通讯)</t>
   </si>
   <si>
     <t>remote_command</t>
@@ -2824,7 +2833,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="110">
+  <cellXfs count="104">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -3105,21 +3114,6 @@
     <xf numFmtId="0" fontId="15" fillId="0" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -3130,9 +3124,6 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -4061,41 +4052,41 @@
   <sheetData>
     <row r="1" ht="21" spans="1:6">
       <c r="A1" s="74" t="s">
-        <v>303</v>
+        <v>306</v>
       </c>
       <c r="B1" s="74" t="s">
-        <v>304</v>
+        <v>307</v>
       </c>
       <c r="C1" s="74" t="s">
-        <v>305</v>
+        <v>308</v>
       </c>
       <c r="D1" s="74" t="s">
-        <v>306</v>
+        <v>309</v>
       </c>
       <c r="E1" s="74" t="s">
-        <v>307</v>
+        <v>310</v>
       </c>
     </row>
     <row r="2" ht="21" spans="1:6">
       <c r="A2" s="74" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
       <c r="B2" s="16" t="s">
-        <v>309</v>
+        <v>312</v>
       </c>
       <c r="C2" s="16" t="s">
-        <v>310</v>
+        <v>313</v>
       </c>
       <c r="D2" s="16" t="s">
-        <v>311</v>
+        <v>314</v>
       </c>
       <c r="E2" s="75" t="s">
-        <v>312</v>
+        <v>315</v>
       </c>
     </row>
     <row r="3" ht="21" spans="1:6">
       <c r="A3" s="74" t="s">
-        <v>313</v>
+        <v>316</v>
       </c>
       <c r="B3" s="16">
         <v>5</v>
@@ -4112,44 +4103,44 @@
     </row>
     <row r="4" ht="21" spans="1:6">
       <c r="A4" s="74" t="s">
-        <v>314</v>
+        <v>317</v>
       </c>
       <c r="B4" s="16" t="s">
-        <v>315</v>
+        <v>318</v>
       </c>
       <c r="C4" s="16" t="s">
-        <v>315</v>
+        <v>318</v>
       </c>
       <c r="D4" s="16" t="s">
-        <v>315</v>
+        <v>318</v>
       </c>
       <c r="E4" s="75" t="s">
-        <v>315</v>
+        <v>318</v>
       </c>
       <c r="F4" t="s">
-        <v>316</v>
+        <v>319</v>
       </c>
     </row>
     <row r="5" ht="21" spans="1:6">
       <c r="A5" s="74" t="s">
-        <v>317</v>
+        <v>320</v>
       </c>
       <c r="B5" s="16" t="s">
-        <v>309</v>
+        <v>312</v>
       </c>
       <c r="C5" s="16" t="s">
-        <v>318</v>
+        <v>321</v>
       </c>
       <c r="D5" s="16" t="s">
-        <v>311</v>
+        <v>314</v>
       </c>
       <c r="E5" s="75" t="s">
-        <v>319</v>
+        <v>322</v>
       </c>
     </row>
     <row r="6" ht="21" spans="1:6">
       <c r="A6" s="74" t="s">
-        <v>313</v>
+        <v>316</v>
       </c>
       <c r="B6" s="16">
         <v>1</v>
@@ -4166,22 +4157,22 @@
     </row>
     <row r="7" ht="21" spans="1:6">
       <c r="A7" s="74" t="s">
-        <v>320</v>
+        <v>323</v>
       </c>
       <c r="B7" s="16" t="s">
-        <v>321</v>
+        <v>324</v>
       </c>
       <c r="C7" s="16" t="s">
-        <v>322</v>
+        <v>325</v>
       </c>
       <c r="D7" s="16"/>
       <c r="E7" s="75" t="s">
-        <v>322</v>
+        <v>325</v>
       </c>
     </row>
     <row r="8" ht="21" spans="1:6">
       <c r="A8" s="74" t="s">
-        <v>313</v>
+        <v>316</v>
       </c>
       <c r="B8" s="75">
         <v>0</v>
@@ -4198,7 +4189,7 @@
     </row>
     <row r="9" ht="21" spans="1:6">
       <c r="A9" s="74" t="s">
-        <v>313</v>
+        <v>316</v>
       </c>
       <c r="B9" s="75">
         <v>0</v>
@@ -4236,13 +4227,13 @@
   <sheetData>
     <row r="1" ht="14.25" spans="1:7">
       <c r="A1" s="53" t="s">
-        <v>323</v>
+        <v>326</v>
       </c>
       <c r="B1" s="54" t="s">
-        <v>324</v>
+        <v>327</v>
       </c>
       <c r="C1" s="55" t="s">
-        <v>325</v>
+        <v>328</v>
       </c>
       <c r="D1" s="56"/>
       <c r="E1" s="57"/>
@@ -4255,16 +4246,16 @@
       <c r="A2" s="59"/>
       <c r="B2" s="60"/>
       <c r="C2" s="61" t="s">
-        <v>326</v>
+        <v>329</v>
       </c>
       <c r="D2" s="61" t="s">
-        <v>327</v>
+        <v>330</v>
       </c>
       <c r="E2" s="62" t="s">
-        <v>328</v>
+        <v>331</v>
       </c>
       <c r="F2" s="62" t="s">
-        <v>327</v>
+        <v>330</v>
       </c>
       <c r="G2" s="63"/>
     </row>
@@ -4273,23 +4264,23 @@
         <v>4000</v>
       </c>
       <c r="B3" s="65" t="s">
-        <v>329</v>
+        <v>332</v>
       </c>
       <c r="C3" s="66" t="s">
-        <v>330</v>
+        <v>333</v>
       </c>
       <c r="D3" s="66"/>
       <c r="E3" s="67"/>
       <c r="F3" s="64"/>
       <c r="G3" s="67" t="s">
-        <v>331</v>
+        <v>334</v>
       </c>
     </row>
     <row r="4" spans="1:7">
       <c r="A4" s="64"/>
       <c r="B4" s="68"/>
       <c r="C4" s="66" t="s">
-        <v>332</v>
+        <v>335</v>
       </c>
       <c r="D4" s="66"/>
       <c r="E4" s="67"/>
@@ -4301,16 +4292,16 @@
         <v>4001</v>
       </c>
       <c r="B5" s="67" t="s">
-        <v>333</v>
+        <v>336</v>
       </c>
       <c r="C5" s="66" t="s">
-        <v>334</v>
+        <v>337</v>
       </c>
       <c r="D5" s="66"/>
       <c r="E5" s="67"/>
       <c r="F5" s="64"/>
       <c r="G5" s="67" t="s">
-        <v>333</v>
+        <v>336</v>
       </c>
     </row>
     <row r="6" spans="1:7">
@@ -4318,23 +4309,23 @@
         <v>4002</v>
       </c>
       <c r="B6" s="70" t="s">
-        <v>335</v>
+        <v>338</v>
       </c>
       <c r="C6" s="66" t="s">
-        <v>336</v>
+        <v>339</v>
       </c>
       <c r="D6" s="66"/>
       <c r="E6" s="67"/>
       <c r="F6" s="64"/>
       <c r="G6" s="69" t="s">
-        <v>335</v>
+        <v>338</v>
       </c>
     </row>
     <row r="7" spans="1:7">
       <c r="A7" s="71"/>
       <c r="B7" s="68"/>
       <c r="C7" s="66" t="s">
-        <v>337</v>
+        <v>340</v>
       </c>
       <c r="D7" s="66"/>
       <c r="E7" s="67"/>
@@ -4345,10 +4336,10 @@
       <c r="A8" s="71"/>
       <c r="B8" s="68"/>
       <c r="C8" s="66" t="s">
-        <v>338</v>
+        <v>341</v>
       </c>
       <c r="D8" s="66" t="s">
-        <v>339</v>
+        <v>342</v>
       </c>
       <c r="E8" s="67"/>
       <c r="F8" s="64"/>
@@ -4358,7 +4349,7 @@
       <c r="A9" s="72"/>
       <c r="B9" s="73"/>
       <c r="C9" s="66" t="s">
-        <v>340</v>
+        <v>343</v>
       </c>
       <c r="D9" s="66"/>
       <c r="E9" s="66"/>
@@ -4370,13 +4361,13 @@
         <v>4003</v>
       </c>
       <c r="B10" s="70" t="s">
-        <v>341</v>
+        <v>344</v>
       </c>
       <c r="C10" s="66" t="s">
-        <v>342</v>
+        <v>345</v>
       </c>
       <c r="D10" s="66" t="s">
-        <v>343</v>
+        <v>346</v>
       </c>
       <c r="E10" s="66"/>
       <c r="F10" s="66"/>
@@ -4386,10 +4377,10 @@
       <c r="A11" s="72"/>
       <c r="B11" s="73"/>
       <c r="C11" s="66" t="s">
-        <v>344</v>
+        <v>347</v>
       </c>
       <c r="D11" s="66" t="s">
-        <v>345</v>
+        <v>348</v>
       </c>
       <c r="E11" s="66"/>
       <c r="F11" s="66"/>
@@ -4400,10 +4391,10 @@
         <v>4004</v>
       </c>
       <c r="B12" s="70" t="s">
-        <v>346</v>
+        <v>349</v>
       </c>
       <c r="C12" s="66" t="s">
-        <v>347</v>
+        <v>350</v>
       </c>
       <c r="D12" s="66"/>
       <c r="E12" s="66"/>
@@ -4414,7 +4405,7 @@
       <c r="A13" s="72"/>
       <c r="B13" s="73"/>
       <c r="C13" s="66" t="s">
-        <v>348</v>
+        <v>351</v>
       </c>
       <c r="D13" s="66"/>
       <c r="E13" s="66"/>
@@ -4426,10 +4417,10 @@
         <v>4005</v>
       </c>
       <c r="B14" s="70" t="s">
-        <v>349</v>
+        <v>352</v>
       </c>
       <c r="C14" s="66" t="s">
-        <v>332</v>
+        <v>335</v>
       </c>
       <c r="D14" s="66"/>
       <c r="E14" s="66"/>
@@ -4440,7 +4431,7 @@
       <c r="A15" s="72"/>
       <c r="B15" s="73"/>
       <c r="C15" s="66" t="s">
-        <v>350</v>
+        <v>353</v>
       </c>
       <c r="D15" s="66"/>
       <c r="E15" s="66"/>
@@ -4452,10 +4443,10 @@
         <v>4006</v>
       </c>
       <c r="B16" s="70" t="s">
-        <v>351</v>
+        <v>354</v>
       </c>
       <c r="C16" s="66" t="s">
-        <v>352</v>
+        <v>355</v>
       </c>
       <c r="D16" s="66"/>
       <c r="E16" s="66"/>
@@ -4466,7 +4457,7 @@
       <c r="A17" s="72"/>
       <c r="B17" s="73"/>
       <c r="C17" s="66" t="s">
-        <v>348</v>
+        <v>351</v>
       </c>
       <c r="D17" s="66"/>
       <c r="E17" s="66"/>
@@ -4478,10 +4469,10 @@
         <v>4007</v>
       </c>
       <c r="B18" s="70" t="s">
-        <v>353</v>
+        <v>356</v>
       </c>
       <c r="C18" s="66" t="s">
-        <v>352</v>
+        <v>355</v>
       </c>
       <c r="D18" s="66"/>
       <c r="E18" s="66"/>
@@ -4492,7 +4483,7 @@
       <c r="A19" s="72"/>
       <c r="B19" s="73"/>
       <c r="C19" s="66" t="s">
-        <v>348</v>
+        <v>351</v>
       </c>
       <c r="D19" s="66"/>
       <c r="E19" s="66"/>
@@ -4504,10 +4495,10 @@
         <v>4008</v>
       </c>
       <c r="B20" s="70" t="s">
-        <v>354</v>
+        <v>357</v>
       </c>
       <c r="C20" s="66" t="s">
-        <v>352</v>
+        <v>355</v>
       </c>
       <c r="D20" s="66"/>
       <c r="E20" s="67"/>
@@ -4518,7 +4509,7 @@
       <c r="A21" s="72"/>
       <c r="B21" s="73"/>
       <c r="C21" s="66" t="s">
-        <v>355</v>
+        <v>358</v>
       </c>
       <c r="D21" s="66"/>
       <c r="E21" s="67"/>
@@ -4578,27 +4569,27 @@
   <sheetData>
     <row r="1" ht="21.75" spans="4:13">
       <c r="D1" s="2" t="s">
-        <v>356</v>
+        <v>359</v>
       </c>
     </row>
     <row r="2" ht="16.5" spans="4:13">
       <c r="D2" s="3" t="s">
-        <v>357</v>
+        <v>360</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>293</v>
+        <v>296</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>358</v>
+        <v>361</v>
       </c>
       <c r="G2" s="5" t="s">
-        <v>292</v>
+        <v>295</v>
       </c>
       <c r="H2" s="6" t="s">
-        <v>359</v>
+        <v>362</v>
       </c>
       <c r="I2" s="4" t="s">
-        <v>293</v>
+        <v>296</v>
       </c>
     </row>
     <row r="3" ht="16.5" spans="4:13">
@@ -4606,7 +4597,7 @@
         <v>1</v>
       </c>
       <c r="E3" s="7" t="s">
-        <v>360</v>
+        <v>363</v>
       </c>
       <c r="F3" s="7">
         <v>1</v>
@@ -4615,10 +4606,10 @@
         <v>1</v>
       </c>
       <c r="H3" s="8" t="s">
-        <v>361</v>
+        <v>364</v>
       </c>
       <c r="I3" s="9" t="s">
-        <v>297</v>
+        <v>300</v>
       </c>
     </row>
     <row r="4" ht="16.5" spans="4:13">
@@ -4627,7 +4618,7 @@
       <c r="F4" s="10"/>
       <c r="G4" s="10"/>
       <c r="H4" s="8" t="s">
-        <v>362</v>
+        <v>365</v>
       </c>
       <c r="I4" s="11"/>
     </row>
@@ -4637,7 +4628,7 @@
       <c r="F5" s="10"/>
       <c r="G5" s="10"/>
       <c r="H5" s="8" t="s">
-        <v>363</v>
+        <v>366</v>
       </c>
       <c r="I5" s="11"/>
     </row>
@@ -4647,7 +4638,7 @@
       <c r="F6" s="10"/>
       <c r="G6" s="10"/>
       <c r="H6" s="8" t="s">
-        <v>364</v>
+        <v>367</v>
       </c>
       <c r="I6" s="11"/>
     </row>
@@ -4657,7 +4648,7 @@
       <c r="F7" s="12"/>
       <c r="G7" s="12"/>
       <c r="H7" s="8" t="s">
-        <v>365</v>
+        <v>368</v>
       </c>
       <c r="I7" s="13"/>
     </row>
@@ -4666,7 +4657,7 @@
         <v>2</v>
       </c>
       <c r="E8" s="7" t="s">
-        <v>366</v>
+        <v>369</v>
       </c>
       <c r="F8" s="7">
         <v>2</v>
@@ -4675,16 +4666,16 @@
         <v>2</v>
       </c>
       <c r="H8" s="8" t="s">
-        <v>361</v>
+        <v>364</v>
       </c>
       <c r="I8" s="9" t="s">
-        <v>295</v>
+        <v>298</v>
       </c>
       <c r="K8" s="14" t="s">
-        <v>367</v>
+        <v>370</v>
       </c>
       <c r="L8" s="4" t="s">
-        <v>293</v>
+        <v>296</v>
       </c>
       <c r="M8" s="15"/>
     </row>
@@ -4694,17 +4685,17 @@
       <c r="F9" s="10"/>
       <c r="G9" s="10"/>
       <c r="H9" s="8" t="s">
-        <v>368</v>
+        <v>371</v>
       </c>
       <c r="I9" s="11"/>
       <c r="K9" s="16">
         <v>1</v>
       </c>
       <c r="L9" s="16" t="s">
-        <v>297</v>
+        <v>300</v>
       </c>
       <c r="M9" s="17" t="s">
-        <v>361</v>
+        <v>364</v>
       </c>
     </row>
     <row r="10" ht="16.5" spans="4:13">
@@ -4713,13 +4704,13 @@
       <c r="F10" s="10"/>
       <c r="G10" s="10"/>
       <c r="H10" s="8" t="s">
-        <v>369</v>
+        <v>372</v>
       </c>
       <c r="I10" s="11"/>
       <c r="K10" s="18"/>
       <c r="L10" s="18"/>
       <c r="M10" s="17" t="s">
-        <v>362</v>
+        <v>365</v>
       </c>
     </row>
     <row r="11" ht="16.5" spans="4:13">
@@ -4728,13 +4719,13 @@
       <c r="F11" s="12"/>
       <c r="G11" s="12"/>
       <c r="H11" s="8" t="s">
-        <v>370</v>
+        <v>373</v>
       </c>
       <c r="I11" s="13"/>
       <c r="K11" s="18"/>
       <c r="L11" s="18"/>
       <c r="M11" s="17" t="s">
-        <v>363</v>
+        <v>366</v>
       </c>
     </row>
     <row r="12" ht="16.5" spans="4:13">
@@ -4742,7 +4733,7 @@
         <v>3</v>
       </c>
       <c r="E12" s="20" t="s">
-        <v>371</v>
+        <v>374</v>
       </c>
       <c r="F12" s="20">
         <v>3</v>
@@ -4751,15 +4742,15 @@
         <v>3</v>
       </c>
       <c r="H12" s="21" t="s">
-        <v>372</v>
+        <v>375</v>
       </c>
       <c r="I12" s="21" t="s">
-        <v>373</v>
+        <v>376</v>
       </c>
       <c r="K12" s="18"/>
       <c r="L12" s="18"/>
       <c r="M12" s="17" t="s">
-        <v>364</v>
+        <v>367</v>
       </c>
     </row>
     <row r="13" ht="16.5" spans="4:13">
@@ -4767,7 +4758,7 @@
         <v>4</v>
       </c>
       <c r="E13" s="22" t="s">
-        <v>374</v>
+        <v>377</v>
       </c>
       <c r="F13" s="22">
         <v>4</v>
@@ -4776,15 +4767,15 @@
         <v>4</v>
       </c>
       <c r="H13" s="24" t="s">
-        <v>375</v>
+        <v>378</v>
       </c>
       <c r="I13" s="24" t="s">
-        <v>376</v>
+        <v>379</v>
       </c>
       <c r="K13" s="19"/>
       <c r="L13" s="19"/>
       <c r="M13" s="25" t="s">
-        <v>365</v>
+        <v>368</v>
       </c>
     </row>
     <row r="14" ht="16.5" spans="4:13">
@@ -4795,19 +4786,19 @@
         <v>5</v>
       </c>
       <c r="H14" s="24" t="s">
-        <v>375</v>
+        <v>378</v>
       </c>
       <c r="I14" s="24" t="s">
-        <v>377</v>
+        <v>380</v>
       </c>
       <c r="K14" s="16">
         <v>2</v>
       </c>
       <c r="L14" s="16" t="s">
-        <v>295</v>
+        <v>298</v>
       </c>
       <c r="M14" s="17" t="s">
-        <v>361</v>
+        <v>364</v>
       </c>
     </row>
     <row r="15" ht="16.5" spans="4:13">
@@ -4815,7 +4806,7 @@
         <v>5</v>
       </c>
       <c r="E15" s="22" t="s">
-        <v>378</v>
+        <v>381</v>
       </c>
       <c r="F15" s="22">
         <v>5</v>
@@ -4824,15 +4815,15 @@
         <v>4</v>
       </c>
       <c r="H15" s="24" t="s">
-        <v>375</v>
+        <v>378</v>
       </c>
       <c r="I15" s="24" t="s">
-        <v>376</v>
+        <v>379</v>
       </c>
       <c r="K15" s="18"/>
       <c r="L15" s="18"/>
       <c r="M15" s="17" t="s">
-        <v>368</v>
+        <v>371</v>
       </c>
     </row>
     <row r="16" ht="16.5" spans="4:13">
@@ -4843,15 +4834,15 @@
         <v>5</v>
       </c>
       <c r="H16" s="24" t="s">
-        <v>375</v>
+        <v>378</v>
       </c>
       <c r="I16" s="24" t="s">
-        <v>377</v>
+        <v>380</v>
       </c>
       <c r="K16" s="18"/>
       <c r="L16" s="18"/>
       <c r="M16" s="17" t="s">
-        <v>369</v>
+        <v>372</v>
       </c>
     </row>
     <row r="17" ht="16.5" spans="4:14">
@@ -4862,15 +4853,15 @@
         <v>6</v>
       </c>
       <c r="H17" s="24" t="s">
-        <v>379</v>
+        <v>382</v>
       </c>
       <c r="I17" s="24" t="s">
-        <v>380</v>
+        <v>383</v>
       </c>
       <c r="K17" s="19"/>
       <c r="L17" s="19"/>
       <c r="M17" s="25" t="s">
-        <v>370</v>
+        <v>373</v>
       </c>
     </row>
     <row r="18" ht="16.5" spans="4:14">
@@ -4878,7 +4869,7 @@
         <v>6</v>
       </c>
       <c r="E18" s="23" t="s">
-        <v>381</v>
+        <v>384</v>
       </c>
       <c r="F18" s="22">
         <v>6</v>
@@ -4887,19 +4878,19 @@
         <v>4</v>
       </c>
       <c r="H18" s="28" t="s">
-        <v>375</v>
+        <v>378</v>
       </c>
       <c r="I18" s="28" t="s">
-        <v>376</v>
+        <v>379</v>
       </c>
       <c r="K18" s="19">
         <v>3</v>
       </c>
       <c r="L18" s="20" t="s">
-        <v>382</v>
+        <v>385</v>
       </c>
       <c r="M18" s="25" t="s">
-        <v>375</v>
+        <v>378</v>
       </c>
     </row>
     <row r="19" ht="16.5" spans="4:14">
@@ -4907,7 +4898,7 @@
         <v>7</v>
       </c>
       <c r="E19" s="23" t="s">
-        <v>383</v>
+        <v>386</v>
       </c>
       <c r="F19" s="26"/>
       <c r="G19" s="26"/>
@@ -4917,10 +4908,10 @@
         <v>4</v>
       </c>
       <c r="L19" s="20" t="s">
-        <v>373</v>
+        <v>376</v>
       </c>
       <c r="M19" s="25" t="s">
-        <v>375</v>
+        <v>378</v>
       </c>
     </row>
     <row r="20" ht="16.5" spans="4:14">
@@ -4928,7 +4919,7 @@
         <v>8</v>
       </c>
       <c r="E20" s="23" t="s">
-        <v>384</v>
+        <v>387</v>
       </c>
       <c r="F20" s="22">
         <v>8</v>
@@ -4937,10 +4928,10 @@
         <v>8</v>
       </c>
       <c r="H20" s="28" t="s">
-        <v>385</v>
+        <v>388</v>
       </c>
       <c r="I20" s="28" t="s">
-        <v>386</v>
+        <v>389</v>
       </c>
     </row>
     <row r="21" ht="16.5" spans="4:14">
@@ -4948,7 +4939,7 @@
         <v>9</v>
       </c>
       <c r="E21" s="23" t="s">
-        <v>387</v>
+        <v>390</v>
       </c>
       <c r="F21" s="26"/>
       <c r="G21" s="26"/>
@@ -4960,7 +4951,7 @@
         <v>10</v>
       </c>
       <c r="E22" s="23" t="s">
-        <v>388</v>
+        <v>391</v>
       </c>
       <c r="F22" s="23">
         <v>10</v>
@@ -4969,10 +4960,10 @@
         <v>10</v>
       </c>
       <c r="H22" s="24" t="s">
-        <v>375</v>
+        <v>378</v>
       </c>
       <c r="I22" s="24" t="s">
-        <v>389</v>
+        <v>392</v>
       </c>
     </row>
     <row r="23" ht="16.5" spans="4:14">
@@ -4999,16 +4990,16 @@
       <c r="H25" s="23"/>
       <c r="I25" s="23"/>
       <c r="K25" s="30" t="s">
-        <v>390</v>
+        <v>393</v>
       </c>
       <c r="L25" s="31" t="s">
-        <v>293</v>
+        <v>296</v>
       </c>
       <c r="M25" s="31" t="s">
-        <v>391</v>
+        <v>394</v>
       </c>
       <c r="N25" s="31" t="s">
-        <v>392</v>
+        <v>395</v>
       </c>
     </row>
     <row r="26" ht="32.25" spans="4:14">
@@ -5019,40 +5010,40 @@
       <c r="H26" s="23"/>
       <c r="I26" s="23"/>
       <c r="K26" s="32" t="s">
-        <v>357</v>
+        <v>360</v>
       </c>
       <c r="L26" s="33" t="s">
-        <v>393</v>
+        <v>396</v>
       </c>
       <c r="M26" s="33"/>
       <c r="N26" s="33" t="s">
-        <v>394</v>
+        <v>397</v>
       </c>
     </row>
     <row r="27" ht="16.5" spans="4:14">
       <c r="D27" s="19"/>
       <c r="E27" s="23" t="s">
-        <v>395</v>
+        <v>398</v>
       </c>
       <c r="F27" s="23"/>
       <c r="G27" s="23"/>
       <c r="H27" s="23"/>
       <c r="I27" s="23"/>
       <c r="K27" s="32" t="s">
-        <v>292</v>
+        <v>295</v>
       </c>
       <c r="L27" s="33" t="s">
-        <v>396</v>
+        <v>399</v>
       </c>
       <c r="M27" s="33"/>
       <c r="N27" s="33" t="s">
-        <v>394</v>
+        <v>397</v>
       </c>
     </row>
     <row r="28" ht="16.5" spans="4:14">
       <c r="D28" s="34"/>
       <c r="E28" s="23" t="s">
-        <v>395</v>
+        <v>398</v>
       </c>
       <c r="F28" s="23"/>
       <c r="G28" s="23"/>
@@ -5062,45 +5053,45 @@
     <row r="37" ht="14.25"/>
     <row r="38" ht="16.5" spans="4:10">
       <c r="D38" s="35" t="s">
-        <v>397</v>
+        <v>400</v>
       </c>
       <c r="E38" s="36" t="s">
-        <v>398</v>
+        <v>401</v>
       </c>
       <c r="F38" s="36" t="s">
-        <v>399</v>
+        <v>402</v>
       </c>
       <c r="G38" s="36" t="s">
-        <v>400</v>
+        <v>403</v>
       </c>
       <c r="H38" s="37" t="s">
+        <v>404</v>
+      </c>
+      <c r="I38" s="38" t="s">
         <v>401</v>
       </c>
-      <c r="I38" s="38" t="s">
-        <v>398</v>
-      </c>
       <c r="J38" s="39" t="s">
-        <v>402</v>
+        <v>405</v>
       </c>
     </row>
     <row r="39" ht="16.5" spans="4:10">
       <c r="D39" s="40" t="s">
-        <v>402</v>
+        <v>405</v>
       </c>
       <c r="E39" s="41" t="s">
-        <v>403</v>
+        <v>406</v>
       </c>
       <c r="F39" s="42" t="s">
-        <v>404</v>
+        <v>407</v>
       </c>
       <c r="G39" s="41" t="s">
-        <v>405</v>
+        <v>408</v>
       </c>
       <c r="H39" s="19">
         <v>1</v>
       </c>
       <c r="I39" s="20" t="s">
-        <v>406</v>
+        <v>409</v>
       </c>
       <c r="J39" s="20">
         <v>2</v>
@@ -5110,14 +5101,14 @@
       <c r="D40" s="43"/>
       <c r="E40" s="44"/>
       <c r="F40" s="42" t="s">
-        <v>407</v>
+        <v>410</v>
       </c>
       <c r="G40" s="44"/>
       <c r="H40" s="19">
         <v>2</v>
       </c>
       <c r="I40" s="20" t="s">
-        <v>408</v>
+        <v>411</v>
       </c>
       <c r="J40" s="20">
         <v>2</v>
@@ -5127,7 +5118,7 @@
       <c r="D41" s="43"/>
       <c r="E41" s="44"/>
       <c r="F41" s="45" t="s">
-        <v>409</v>
+        <v>412</v>
       </c>
       <c r="G41" s="44"/>
     </row>
@@ -5135,7 +5126,7 @@
       <c r="D42" s="43"/>
       <c r="E42" s="44"/>
       <c r="F42" s="46" t="s">
-        <v>410</v>
+        <v>413</v>
       </c>
       <c r="G42" s="44"/>
     </row>
@@ -5143,7 +5134,7 @@
       <c r="D43" s="43"/>
       <c r="E43" s="44"/>
       <c r="F43" s="46" t="s">
-        <v>411</v>
+        <v>414</v>
       </c>
       <c r="G43" s="44"/>
     </row>
@@ -5151,7 +5142,7 @@
       <c r="D44" s="43"/>
       <c r="E44" s="44"/>
       <c r="F44" s="46" t="s">
-        <v>412</v>
+        <v>415</v>
       </c>
       <c r="G44" s="44"/>
     </row>
@@ -5159,7 +5150,7 @@
       <c r="D45" s="43"/>
       <c r="E45" s="44"/>
       <c r="F45" s="46" t="s">
-        <v>413</v>
+        <v>416</v>
       </c>
       <c r="G45" s="44"/>
     </row>
@@ -5167,7 +5158,7 @@
       <c r="D46" s="43"/>
       <c r="E46" s="44"/>
       <c r="F46" s="46" t="s">
-        <v>414</v>
+        <v>417</v>
       </c>
       <c r="G46" s="44"/>
     </row>
@@ -5175,7 +5166,7 @@
       <c r="D47" s="43"/>
       <c r="E47" s="44"/>
       <c r="F47" s="46" t="s">
-        <v>415</v>
+        <v>418</v>
       </c>
       <c r="G47" s="44"/>
     </row>
@@ -5183,7 +5174,7 @@
       <c r="D48" s="43"/>
       <c r="E48" s="44"/>
       <c r="F48" s="46" t="s">
-        <v>416</v>
+        <v>419</v>
       </c>
       <c r="G48" s="44"/>
     </row>
@@ -5191,7 +5182,7 @@
       <c r="D49" s="43"/>
       <c r="E49" s="44"/>
       <c r="F49" s="46" t="s">
-        <v>417</v>
+        <v>420</v>
       </c>
       <c r="G49" s="44"/>
     </row>
@@ -5199,7 +5190,7 @@
       <c r="D50" s="43"/>
       <c r="E50" s="44"/>
       <c r="F50" s="46" t="s">
-        <v>418</v>
+        <v>421</v>
       </c>
       <c r="G50" s="44"/>
     </row>
@@ -5207,7 +5198,7 @@
       <c r="D51" s="43"/>
       <c r="E51" s="44"/>
       <c r="F51" s="46" t="s">
-        <v>419</v>
+        <v>422</v>
       </c>
       <c r="G51" s="44"/>
     </row>
@@ -5215,23 +5206,23 @@
       <c r="D52" s="47"/>
       <c r="E52" s="48"/>
       <c r="F52" s="49" t="s">
-        <v>420</v>
+        <v>423</v>
       </c>
       <c r="G52" s="48"/>
     </row>
     <row r="53" ht="21" spans="4:7">
       <c r="D53" s="50" t="s">
-        <v>421</v>
+        <v>424</v>
       </c>
     </row>
     <row r="54" ht="15.75" spans="4:7">
       <c r="D54" s="51" t="s">
-        <v>404</v>
+        <v>407</v>
       </c>
     </row>
     <row r="55" ht="15.75" spans="4:7">
       <c r="D55" s="52" t="s">
-        <v>422</v>
+        <v>425</v>
       </c>
     </row>
   </sheetData>
@@ -5291,176 +5282,176 @@
   </cols>
   <sheetData>
     <row r="1" ht="33" customHeight="1" spans="1:8">
-      <c r="A1" s="107" t="s">
+      <c r="A1" s="101" t="s">
         <v>98</v>
       </c>
-      <c r="B1" s="107" t="s">
+      <c r="B1" s="101" t="s">
         <v>99</v>
       </c>
-      <c r="C1" s="107" t="s">
+      <c r="C1" s="101" t="s">
         <v>100</v>
       </c>
-      <c r="D1" s="107" t="s">
+      <c r="D1" s="101" t="s">
         <v>101</v>
       </c>
-      <c r="E1" s="107" t="s">
+      <c r="E1" s="101" t="s">
         <v>102</v>
       </c>
-      <c r="F1" s="107" t="s">
+      <c r="F1" s="101" t="s">
         <v>103</v>
       </c>
-      <c r="G1" s="107" t="s">
+      <c r="G1" s="101" t="s">
         <v>104</v>
       </c>
-      <c r="H1" s="107" t="s">
+      <c r="H1" s="101" t="s">
         <v>105</v>
       </c>
     </row>
-    <row r="2" s="106" customFormat="1" ht="75" spans="1:8">
-      <c r="A2" s="108">
+    <row r="2" s="100" customFormat="1" ht="75" spans="1:8">
+      <c r="A2" s="102">
         <v>5001</v>
       </c>
-      <c r="B2" s="108" t="s">
+      <c r="B2" s="102" t="s">
         <v>106</v>
       </c>
-      <c r="C2" s="109" t="s">
+      <c r="C2" s="103" t="s">
         <v>107</v>
       </c>
-      <c r="D2" s="108">
+      <c r="D2" s="102">
         <v>1</v>
       </c>
-      <c r="E2" s="101">
+      <c r="E2" s="96">
         <v>501</v>
       </c>
-      <c r="F2" s="101" t="s">
+      <c r="F2" s="96" t="s">
         <v>108</v>
       </c>
-      <c r="G2" s="101" t="s">
+      <c r="G2" s="96" t="s">
         <v>109</v>
       </c>
-      <c r="H2" s="102" t="s">
+      <c r="H2" s="97" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="3" s="106" customFormat="1" ht="75" spans="1:8">
-      <c r="A3" s="108">
+    <row r="3" s="100" customFormat="1" ht="75" spans="1:8">
+      <c r="A3" s="102">
         <v>5002</v>
       </c>
-      <c r="B3" s="108" t="s">
+      <c r="B3" s="102" t="s">
         <v>111</v>
       </c>
-      <c r="C3" s="109" t="s">
+      <c r="C3" s="103" t="s">
         <v>112</v>
       </c>
-      <c r="D3" s="108">
+      <c r="D3" s="102">
         <v>2</v>
       </c>
-      <c r="E3" s="101">
+      <c r="E3" s="96">
         <v>501</v>
       </c>
-      <c r="F3" s="101" t="s">
+      <c r="F3" s="96" t="s">
         <v>108</v>
       </c>
-      <c r="G3" s="101" t="s">
+      <c r="G3" s="96" t="s">
         <v>109</v>
       </c>
-      <c r="H3" s="102" t="s">
+      <c r="H3" s="97" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="4" s="106" customFormat="1" ht="75" spans="1:8">
-      <c r="A4" s="108">
+    <row r="4" s="100" customFormat="1" ht="75" spans="1:8">
+      <c r="A4" s="102">
         <v>5003</v>
       </c>
-      <c r="B4" s="108" t="s">
+      <c r="B4" s="102" t="s">
         <v>113</v>
       </c>
-      <c r="C4" s="109" t="s">
+      <c r="C4" s="103" t="s">
         <v>114</v>
       </c>
-      <c r="D4" s="108">
+      <c r="D4" s="102">
         <v>3</v>
       </c>
-      <c r="E4" s="101">
+      <c r="E4" s="96">
         <v>501</v>
       </c>
-      <c r="F4" s="101" t="s">
+      <c r="F4" s="96" t="s">
         <v>108</v>
       </c>
-      <c r="G4" s="101" t="s">
+      <c r="G4" s="96" t="s">
         <v>109</v>
       </c>
-      <c r="H4" s="102" t="s">
+      <c r="H4" s="97" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="5" s="106" customFormat="1" ht="75" spans="1:8">
-      <c r="A5" s="108">
+    <row r="5" s="100" customFormat="1" ht="75" spans="1:8">
+      <c r="A5" s="102">
         <v>5004</v>
       </c>
-      <c r="B5" s="108" t="s">
+      <c r="B5" s="102" t="s">
         <v>115</v>
       </c>
-      <c r="C5" s="109" t="s">
+      <c r="C5" s="103" t="s">
         <v>116</v>
       </c>
-      <c r="D5" s="108">
+      <c r="D5" s="102">
         <v>4</v>
       </c>
-      <c r="E5" s="101">
+      <c r="E5" s="96">
         <v>501</v>
       </c>
-      <c r="F5" s="101" t="s">
+      <c r="F5" s="96" t="s">
         <v>108</v>
       </c>
-      <c r="G5" s="101" t="s">
+      <c r="G5" s="96" t="s">
         <v>109</v>
       </c>
-      <c r="H5" s="102" t="s">
+      <c r="H5" s="97" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="6" s="106" customFormat="1" ht="56.25" spans="1:8">
-      <c r="A6" s="108">
+    <row r="6" s="100" customFormat="1" ht="56.25" spans="1:8">
+      <c r="A6" s="102">
         <v>5005</v>
       </c>
-      <c r="B6" s="108" t="s">
+      <c r="B6" s="102" t="s">
         <v>117</v>
       </c>
-      <c r="C6" s="109" t="s">
+      <c r="C6" s="103" t="s">
         <v>118</v>
       </c>
-      <c r="D6" s="108">
+      <c r="D6" s="102">
         <v>5</v>
       </c>
-      <c r="E6" s="108">
+      <c r="E6" s="102">
         <v>502</v>
       </c>
-      <c r="F6" s="108" t="s">
+      <c r="F6" s="102" t="s">
         <v>119</v>
       </c>
-      <c r="G6" s="108" t="s">
+      <c r="G6" s="102" t="s">
         <v>109</v>
       </c>
-      <c r="H6" s="102" t="s">
+      <c r="H6" s="97" t="s">
         <v>120</v>
       </c>
     </row>
-    <row r="7" s="106" customFormat="1" ht="20.25" spans="1:8">
-      <c r="A7" s="108"/>
-      <c r="B7" s="108"/>
-      <c r="C7" s="109"/>
-      <c r="D7" s="108"/>
-      <c r="E7" s="101">
+    <row r="7" s="100" customFormat="1" ht="20.25" spans="1:8">
+      <c r="A7" s="102"/>
+      <c r="B7" s="102"/>
+      <c r="C7" s="103"/>
+      <c r="D7" s="102"/>
+      <c r="E7" s="96">
         <v>503</v>
       </c>
-      <c r="F7" s="101" t="s">
+      <c r="F7" s="96" t="s">
         <v>121</v>
       </c>
-      <c r="G7" s="101" t="s">
+      <c r="G7" s="96" t="s">
         <v>109</v>
       </c>
-      <c r="H7" s="109" t="s">
+      <c r="H7" s="103" t="s">
         <v>122</v>
       </c>
     </row>
@@ -5484,13 +5475,13 @@
   <dimension ref="A1:G20"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="18.75" outlineLevelCol="6"/>
   <cols>
-    <col min="1" max="1" width="6.66666666666667" style="100" customWidth="1"/>
-    <col min="2" max="2" width="29.8833333333333" style="100" customWidth="1"/>
-    <col min="3" max="3" width="16" style="100" customWidth="1"/>
-    <col min="4" max="5" width="25.125" style="100" customWidth="1"/>
-    <col min="6" max="6" width="57.5" style="100" customWidth="1"/>
-    <col min="7" max="7" width="36.375" style="100" customWidth="1"/>
-    <col min="8" max="16384" width="9" style="100"/>
+    <col min="1" max="1" width="6.66666666666667" style="95" customWidth="1"/>
+    <col min="2" max="2" width="29.8833333333333" style="95" customWidth="1"/>
+    <col min="3" max="3" width="16" style="95" customWidth="1"/>
+    <col min="4" max="5" width="25.125" style="95" customWidth="1"/>
+    <col min="6" max="6" width="57.5" style="95" customWidth="1"/>
+    <col min="7" max="7" width="36.375" style="95" customWidth="1"/>
+    <col min="8" max="16384" width="9" style="95"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
@@ -5513,322 +5504,322 @@
         <v>127</v>
       </c>
     </row>
-    <row r="2" s="99" customFormat="1" ht="75" spans="1:7">
-      <c r="A2" s="101">
+    <row r="2" s="94" customFormat="1" ht="75" spans="1:7">
+      <c r="A2" s="96">
         <v>501</v>
       </c>
-      <c r="B2" s="101" t="s">
+      <c r="B2" s="96" t="s">
         <v>108</v>
       </c>
-      <c r="C2" s="101" t="s">
+      <c r="C2" s="96" t="s">
         <v>109</v>
       </c>
-      <c r="D2" s="101"/>
-      <c r="E2" s="101"/>
-      <c r="F2" s="102" t="s">
+      <c r="D2" s="96"/>
+      <c r="E2" s="96"/>
+      <c r="F2" s="97" t="s">
         <v>110</v>
       </c>
-      <c r="G2" s="100"/>
-    </row>
-    <row r="3" s="100" customFormat="1" ht="56.25" spans="1:7">
-      <c r="A3" s="101">
+      <c r="G2" s="95"/>
+    </row>
+    <row r="3" s="95" customFormat="1" ht="56.25" spans="1:7">
+      <c r="A3" s="96">
         <v>502</v>
       </c>
-      <c r="B3" s="101" t="s">
+      <c r="B3" s="96" t="s">
         <v>119</v>
       </c>
-      <c r="C3" s="101" t="s">
+      <c r="C3" s="96" t="s">
         <v>109</v>
       </c>
-      <c r="D3" s="101"/>
-      <c r="E3" s="101"/>
-      <c r="F3" s="102" t="s">
+      <c r="D3" s="96"/>
+      <c r="E3" s="96"/>
+      <c r="F3" s="97" t="s">
         <v>120</v>
       </c>
     </row>
-    <row r="4" s="100" customFormat="1" spans="1:7">
-      <c r="A4" s="101">
+    <row r="4" s="95" customFormat="1" spans="1:7">
+      <c r="A4" s="96">
         <v>503</v>
       </c>
-      <c r="B4" s="101" t="s">
+      <c r="B4" s="96" t="s">
         <v>121</v>
       </c>
-      <c r="C4" s="101" t="s">
+      <c r="C4" s="96" t="s">
         <v>109</v>
       </c>
-      <c r="D4" s="101"/>
-      <c r="E4" s="101"/>
-      <c r="F4" s="101" t="s">
+      <c r="D4" s="96"/>
+      <c r="E4" s="96"/>
+      <c r="F4" s="96" t="s">
         <v>122</v>
       </c>
     </row>
-    <row r="5" s="100" customFormat="1" spans="1:7">
-      <c r="A5" s="101">
+    <row r="5" s="95" customFormat="1" spans="1:7">
+      <c r="A5" s="96">
         <v>504</v>
       </c>
-      <c r="B5" s="101" t="s">
+      <c r="B5" s="96" t="s">
         <v>128</v>
       </c>
-      <c r="C5" s="101" t="s">
+      <c r="C5" s="96" t="s">
         <v>129</v>
       </c>
-      <c r="D5" s="101"/>
-      <c r="E5" s="101"/>
-      <c r="F5" s="101" t="s">
+      <c r="D5" s="96"/>
+      <c r="E5" s="96"/>
+      <c r="F5" s="96" t="s">
         <v>130</v>
       </c>
     </row>
-    <row r="6" s="100" customFormat="1" spans="1:7">
-      <c r="A6" s="101">
+    <row r="6" s="95" customFormat="1" spans="1:7">
+      <c r="A6" s="96">
         <v>505</v>
       </c>
-      <c r="B6" s="101" t="s">
+      <c r="B6" s="96" t="s">
         <v>131</v>
       </c>
-      <c r="C6" s="101" t="s">
+      <c r="C6" s="96" t="s">
         <v>129</v>
       </c>
-      <c r="D6" s="101"/>
-      <c r="E6" s="102" t="s">
+      <c r="D6" s="96"/>
+      <c r="E6" s="97" t="s">
         <v>132</v>
       </c>
-      <c r="F6" s="101" t="s">
+      <c r="F6" s="96" t="s">
         <v>133</v>
       </c>
     </row>
-    <row r="7" s="100" customFormat="1" spans="1:7">
-      <c r="A7" s="101">
+    <row r="7" s="95" customFormat="1" spans="1:7">
+      <c r="A7" s="96">
         <v>506</v>
       </c>
-      <c r="B7" s="101" t="s">
+      <c r="B7" s="96" t="s">
         <v>134</v>
       </c>
-      <c r="C7" s="101" t="s">
+      <c r="C7" s="96" t="s">
         <v>129</v>
       </c>
-      <c r="D7" s="101"/>
-      <c r="E7" s="102"/>
-      <c r="F7" s="101" t="s">
+      <c r="D7" s="96"/>
+      <c r="E7" s="97"/>
+      <c r="F7" s="96" t="s">
         <v>135</v>
       </c>
     </row>
-    <row r="8" s="100" customFormat="1" spans="1:7">
-      <c r="A8" s="101">
+    <row r="8" s="95" customFormat="1" spans="1:7">
+      <c r="A8" s="96">
         <v>511</v>
       </c>
-      <c r="B8" s="101" t="s">
+      <c r="B8" s="96" t="s">
         <v>136</v>
       </c>
-      <c r="C8" s="101" t="s">
+      <c r="C8" s="96" t="s">
         <v>129</v>
       </c>
-      <c r="D8" s="101"/>
-      <c r="E8" s="102"/>
-      <c r="F8" s="101" t="s">
+      <c r="D8" s="96"/>
+      <c r="E8" s="97"/>
+      <c r="F8" s="96" t="s">
         <v>137</v>
       </c>
     </row>
-    <row r="9" s="100" customFormat="1" spans="1:7">
-      <c r="A9" s="101">
+    <row r="9" s="95" customFormat="1" spans="1:7">
+      <c r="A9" s="96">
         <v>512</v>
       </c>
-      <c r="B9" s="101" t="s">
+      <c r="B9" s="96" t="s">
         <v>138</v>
       </c>
-      <c r="C9" s="101" t="s">
+      <c r="C9" s="96" t="s">
         <v>109</v>
       </c>
-      <c r="D9" s="101"/>
-      <c r="E9" s="102"/>
-      <c r="F9" s="101" t="s">
+      <c r="D9" s="96"/>
+      <c r="E9" s="97"/>
+      <c r="F9" s="96" t="s">
         <v>139</v>
       </c>
     </row>
-    <row r="10" s="100" customFormat="1" spans="1:7">
-      <c r="A10" s="101">
+    <row r="10" s="95" customFormat="1" spans="1:7">
+      <c r="A10" s="96">
         <v>513</v>
       </c>
-      <c r="B10" s="101" t="s">
+      <c r="B10" s="96" t="s">
         <v>140</v>
       </c>
-      <c r="C10" s="101" t="s">
+      <c r="C10" s="96" t="s">
         <v>109</v>
       </c>
-      <c r="D10" s="101"/>
-      <c r="E10" s="102"/>
-      <c r="F10" s="101" t="s">
+      <c r="D10" s="96"/>
+      <c r="E10" s="97"/>
+      <c r="F10" s="96" t="s">
         <v>141</v>
       </c>
     </row>
-    <row r="11" s="100" customFormat="1" spans="1:7">
-      <c r="A11" s="101">
+    <row r="11" s="95" customFormat="1" spans="1:7">
+      <c r="A11" s="96">
         <v>514</v>
       </c>
-      <c r="B11" s="101" t="s">
+      <c r="B11" s="96" t="s">
         <v>142</v>
       </c>
-      <c r="C11" s="101" t="s">
+      <c r="C11" s="96" t="s">
         <v>109</v>
       </c>
-      <c r="D11" s="101"/>
-      <c r="E11" s="102">
+      <c r="D11" s="96"/>
+      <c r="E11" s="97">
         <v>1</v>
       </c>
-      <c r="F11" s="101" t="s">
+      <c r="F11" s="96" t="s">
         <v>143</v>
       </c>
     </row>
-    <row r="12" s="100" customFormat="1" spans="1:7">
-      <c r="A12" s="101">
+    <row r="12" s="95" customFormat="1" spans="1:7">
+      <c r="A12" s="96">
         <v>515</v>
       </c>
-      <c r="B12" s="101" t="s">
+      <c r="B12" s="96" t="s">
         <v>144</v>
       </c>
-      <c r="C12" s="101" t="s">
+      <c r="C12" s="96" t="s">
         <v>109</v>
       </c>
-      <c r="D12" s="101"/>
-      <c r="E12" s="102">
+      <c r="D12" s="96"/>
+      <c r="E12" s="97">
         <v>2</v>
       </c>
-      <c r="F12" s="101" t="s">
+      <c r="F12" s="96" t="s">
         <v>145</v>
       </c>
     </row>
-    <row r="13" s="99" customFormat="1" spans="1:7">
-      <c r="A13" s="101">
+    <row r="13" s="94" customFormat="1" spans="1:7">
+      <c r="A13" s="96">
         <v>516</v>
       </c>
-      <c r="B13" s="101" t="s">
+      <c r="B13" s="96" t="s">
         <v>146</v>
       </c>
-      <c r="C13" s="101" t="s">
+      <c r="C13" s="96" t="s">
         <v>109</v>
       </c>
-      <c r="D13" s="101"/>
-      <c r="E13" s="102">
+      <c r="D13" s="96"/>
+      <c r="E13" s="97">
         <v>3</v>
       </c>
-      <c r="F13" s="101" t="s">
+      <c r="F13" s="96" t="s">
         <v>147</v>
       </c>
-      <c r="G13" s="100"/>
-    </row>
-    <row r="14" s="100" customFormat="1" spans="1:7">
-      <c r="A14" s="101">
+      <c r="G13" s="95"/>
+    </row>
+    <row r="14" s="95" customFormat="1" spans="1:7">
+      <c r="A14" s="96">
         <v>521</v>
       </c>
-      <c r="B14" s="101" t="s">
+      <c r="B14" s="96" t="s">
         <v>148</v>
       </c>
-      <c r="C14" s="101" t="s">
+      <c r="C14" s="96" t="s">
         <v>109</v>
       </c>
-      <c r="D14" s="101"/>
-      <c r="E14" s="102"/>
-      <c r="F14" s="102" t="s">
+      <c r="D14" s="96"/>
+      <c r="E14" s="97"/>
+      <c r="F14" s="97" t="s">
         <v>149</v>
       </c>
     </row>
-    <row r="15" s="100" customFormat="1" spans="1:7">
-      <c r="A15" s="101">
+    <row r="15" s="95" customFormat="1" spans="1:7">
+      <c r="A15" s="96">
         <v>522</v>
       </c>
-      <c r="B15" s="101" t="s">
+      <c r="B15" s="96" t="s">
         <v>150</v>
       </c>
-      <c r="C15" s="101" t="s">
+      <c r="C15" s="96" t="s">
         <v>129</v>
       </c>
-      <c r="D15" s="101"/>
-      <c r="E15" s="102"/>
-      <c r="F15" s="102" t="s">
+      <c r="D15" s="96"/>
+      <c r="E15" s="97"/>
+      <c r="F15" s="97" t="s">
         <v>151</v>
       </c>
     </row>
-    <row r="16" s="100" customFormat="1" spans="1:7">
-      <c r="A16" s="101">
+    <row r="16" s="95" customFormat="1" spans="1:7">
+      <c r="A16" s="96">
         <v>523</v>
       </c>
-      <c r="B16" s="101" t="s">
+      <c r="B16" s="96" t="s">
         <v>152</v>
       </c>
-      <c r="C16" s="101" t="s">
+      <c r="C16" s="96" t="s">
         <v>109</v>
       </c>
-      <c r="D16" s="101"/>
-      <c r="E16" s="102"/>
-      <c r="F16" s="102" t="s">
+      <c r="D16" s="96"/>
+      <c r="E16" s="97"/>
+      <c r="F16" s="97" t="s">
         <v>153</v>
       </c>
     </row>
-    <row r="17" s="100" customFormat="1" spans="1:7">
-      <c r="A17" s="101">
+    <row r="17" s="95" customFormat="1" spans="1:7">
+      <c r="A17" s="96">
         <v>524</v>
       </c>
-      <c r="B17" s="101" t="s">
+      <c r="B17" s="96" t="s">
         <v>154</v>
       </c>
-      <c r="C17" s="101" t="s">
+      <c r="C17" s="96" t="s">
         <v>129</v>
       </c>
-      <c r="D17" s="101"/>
-      <c r="E17" s="102"/>
-      <c r="F17" s="102" t="s">
+      <c r="D17" s="96"/>
+      <c r="E17" s="97"/>
+      <c r="F17" s="97" t="s">
         <v>155</v>
       </c>
     </row>
-    <row r="18" s="100" customFormat="1" spans="1:7">
-      <c r="A18" s="101">
+    <row r="18" s="95" customFormat="1" spans="1:7">
+      <c r="A18" s="96">
         <v>525</v>
       </c>
-      <c r="B18" s="101" t="s">
+      <c r="B18" s="96" t="s">
         <v>156</v>
       </c>
-      <c r="C18" s="101" t="s">
+      <c r="C18" s="96" t="s">
         <v>109</v>
       </c>
-      <c r="D18" s="101"/>
-      <c r="E18" s="102">
+      <c r="D18" s="96"/>
+      <c r="E18" s="97">
         <v>2</v>
       </c>
-      <c r="F18" s="102" t="s">
+      <c r="F18" s="97" t="s">
         <v>157</v>
       </c>
     </row>
-    <row r="19" s="100" customFormat="1" spans="1:7">
-      <c r="A19" s="101">
+    <row r="19" s="95" customFormat="1" spans="1:7">
+      <c r="A19" s="96">
         <v>526</v>
       </c>
-      <c r="B19" s="101" t="s">
+      <c r="B19" s="96" t="s">
         <v>158</v>
       </c>
-      <c r="C19" s="101" t="s">
+      <c r="C19" s="96" t="s">
         <v>109</v>
       </c>
-      <c r="D19" s="101"/>
-      <c r="E19" s="103">
+      <c r="D19" s="96"/>
+      <c r="E19" s="93">
         <v>0</v>
       </c>
-      <c r="F19" s="101" t="s">
+      <c r="F19" s="96" t="s">
         <v>159</v>
       </c>
-      <c r="G19" s="104"/>
+      <c r="G19" s="98"/>
     </row>
     <row r="20" spans="1:7">
-      <c r="A20" s="105">
+      <c r="A20" s="99">
         <v>527</v>
       </c>
-      <c r="B20" s="105" t="s">
+      <c r="B20" s="99" t="s">
         <v>160</v>
       </c>
-      <c r="C20" s="105" t="s">
+      <c r="C20" s="99" t="s">
         <v>109</v>
       </c>
-      <c r="D20" s="105"/>
-      <c r="E20" s="105"/>
-      <c r="F20" s="105" t="s">
+      <c r="D20" s="99"/>
+      <c r="E20" s="99"/>
+      <c r="F20" s="99" t="s">
         <v>161</v>
       </c>
     </row>
@@ -5845,12 +5836,12 @@
   <dimension ref="A1:F14"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" outlineLevelCol="5"/>
   <cols>
-    <col min="1" max="1" width="8.84166666666667" style="97" customWidth="1"/>
-    <col min="2" max="2" width="30.8666666666667" style="97" customWidth="1"/>
-    <col min="3" max="3" width="12.3333333333333" style="97" customWidth="1"/>
-    <col min="4" max="5" width="18.625" style="97" customWidth="1"/>
-    <col min="6" max="6" width="36.925" style="97" customWidth="1"/>
-    <col min="7" max="16384" width="9" style="97"/>
+    <col min="1" max="1" width="8.84166666666667" style="81" customWidth="1"/>
+    <col min="2" max="2" width="30.8666666666667" style="81" customWidth="1"/>
+    <col min="3" max="3" width="12.3333333333333" style="81" customWidth="1"/>
+    <col min="4" max="5" width="18.625" style="81" customWidth="1"/>
+    <col min="6" max="6" width="36.925" style="81" customWidth="1"/>
+    <col min="7" max="16384" width="9" style="81"/>
   </cols>
   <sheetData>
     <row r="1" ht="19" customHeight="1" spans="1:6">
@@ -5874,218 +5865,218 @@
       </c>
     </row>
     <row r="2" spans="1:6">
-      <c r="A2" s="98">
+      <c r="A2" s="86">
         <v>601</v>
       </c>
-      <c r="B2" s="98" t="s">
+      <c r="B2" s="86" t="s">
         <v>164</v>
       </c>
-      <c r="C2" s="98" t="s">
+      <c r="C2" s="86" t="s">
         <v>129</v>
       </c>
-      <c r="D2" s="98"/>
-      <c r="E2" s="98"/>
-      <c r="F2" s="98" t="s">
+      <c r="D2" s="86"/>
+      <c r="E2" s="86"/>
+      <c r="F2" s="86" t="s">
         <v>165</v>
       </c>
     </row>
     <row r="3" spans="1:6">
-      <c r="A3" s="98">
+      <c r="A3" s="86">
         <v>602</v>
       </c>
-      <c r="B3" s="98" t="s">
+      <c r="B3" s="86" t="s">
         <v>166</v>
       </c>
-      <c r="C3" s="98" t="s">
+      <c r="C3" s="86" t="s">
         <v>167</v>
       </c>
-      <c r="D3" s="98" t="s">
+      <c r="D3" s="86" t="s">
         <v>129</v>
       </c>
-      <c r="E3" s="98"/>
-      <c r="F3" s="98" t="s">
+      <c r="E3" s="86"/>
+      <c r="F3" s="86" t="s">
         <v>168</v>
       </c>
     </row>
     <row r="4" spans="1:6">
-      <c r="A4" s="98">
+      <c r="A4" s="86">
         <v>603</v>
       </c>
-      <c r="B4" s="98" t="s">
+      <c r="B4" s="86" t="s">
         <v>169</v>
       </c>
-      <c r="C4" s="98" t="s">
+      <c r="C4" s="86" t="s">
         <v>167</v>
       </c>
-      <c r="D4" s="98" t="s">
+      <c r="D4" s="86" t="s">
         <v>109</v>
       </c>
-      <c r="E4" s="98"/>
-      <c r="F4" s="98" t="s">
+      <c r="E4" s="86"/>
+      <c r="F4" s="86" t="s">
         <v>170</v>
       </c>
     </row>
     <row r="5" spans="1:6">
-      <c r="A5" s="98">
+      <c r="A5" s="86">
         <v>604</v>
       </c>
-      <c r="B5" s="98" t="s">
+      <c r="B5" s="86" t="s">
         <v>171</v>
       </c>
-      <c r="C5" s="98" t="s">
+      <c r="C5" s="86" t="s">
         <v>109</v>
       </c>
-      <c r="D5" s="98"/>
-      <c r="E5" s="98"/>
-      <c r="F5" s="98" t="s">
+      <c r="D5" s="86"/>
+      <c r="E5" s="86"/>
+      <c r="F5" s="86" t="s">
         <v>172</v>
       </c>
     </row>
     <row r="6" spans="1:6">
-      <c r="A6" s="98">
+      <c r="A6" s="86">
         <v>605</v>
       </c>
-      <c r="B6" s="98" t="s">
+      <c r="B6" s="86" t="s">
         <v>173</v>
       </c>
-      <c r="C6" s="98" t="s">
+      <c r="C6" s="86" t="s">
         <v>174</v>
       </c>
-      <c r="D6" s="98"/>
-      <c r="E6" s="98"/>
-      <c r="F6" s="98" t="s">
+      <c r="D6" s="86"/>
+      <c r="E6" s="86"/>
+      <c r="F6" s="86" t="s">
         <v>175</v>
       </c>
     </row>
     <row r="7" spans="1:6">
-      <c r="A7" s="98">
+      <c r="A7" s="86">
         <v>611</v>
       </c>
-      <c r="B7" s="98" t="s">
+      <c r="B7" s="86" t="s">
         <v>176</v>
       </c>
-      <c r="C7" s="98" t="s">
+      <c r="C7" s="86" t="s">
         <v>129</v>
       </c>
-      <c r="D7" s="98"/>
-      <c r="E7" s="98"/>
-      <c r="F7" s="98" t="s">
+      <c r="D7" s="86"/>
+      <c r="E7" s="86"/>
+      <c r="F7" s="86" t="s">
         <v>177</v>
       </c>
     </row>
     <row r="8" spans="1:6">
-      <c r="A8" s="98">
+      <c r="A8" s="86">
         <v>612</v>
       </c>
-      <c r="B8" s="98" t="s">
+      <c r="B8" s="86" t="s">
         <v>178</v>
       </c>
-      <c r="C8" s="98" t="s">
+      <c r="C8" s="86" t="s">
         <v>167</v>
       </c>
-      <c r="D8" s="98" t="s">
+      <c r="D8" s="86" t="s">
         <v>129</v>
       </c>
-      <c r="E8" s="98"/>
-      <c r="F8" s="98" t="s">
+      <c r="E8" s="86"/>
+      <c r="F8" s="86" t="s">
         <v>179</v>
       </c>
     </row>
     <row r="9" spans="1:6">
-      <c r="A9" s="98">
+      <c r="A9" s="86">
         <v>613</v>
       </c>
-      <c r="B9" s="98" t="s">
+      <c r="B9" s="86" t="s">
         <v>180</v>
       </c>
-      <c r="C9" s="98" t="s">
+      <c r="C9" s="86" t="s">
         <v>167</v>
       </c>
-      <c r="D9" s="98" t="s">
+      <c r="D9" s="86" t="s">
         <v>109</v>
       </c>
-      <c r="E9" s="98"/>
-      <c r="F9" s="98" t="s">
+      <c r="E9" s="86"/>
+      <c r="F9" s="86" t="s">
         <v>181</v>
       </c>
     </row>
     <row r="10" spans="1:6">
-      <c r="A10" s="98">
+      <c r="A10" s="86">
         <v>614</v>
       </c>
-      <c r="B10" s="98" t="s">
+      <c r="B10" s="86" t="s">
         <v>182</v>
       </c>
-      <c r="C10" s="98" t="s">
+      <c r="C10" s="86" t="s">
         <v>109</v>
       </c>
-      <c r="D10" s="98"/>
-      <c r="E10" s="98"/>
-      <c r="F10" s="98" t="s">
+      <c r="D10" s="86"/>
+      <c r="E10" s="86"/>
+      <c r="F10" s="86" t="s">
         <v>183</v>
       </c>
     </row>
     <row r="11" spans="1:6">
-      <c r="A11" s="98">
+      <c r="A11" s="86">
         <v>615</v>
       </c>
-      <c r="B11" s="98" t="s">
+      <c r="B11" s="86" t="s">
         <v>184</v>
       </c>
-      <c r="C11" s="98" t="s">
+      <c r="C11" s="86" t="s">
         <v>174</v>
       </c>
-      <c r="D11" s="98"/>
-      <c r="E11" s="98"/>
-      <c r="F11" s="98" t="s">
+      <c r="D11" s="86"/>
+      <c r="E11" s="86"/>
+      <c r="F11" s="86" t="s">
         <v>185</v>
       </c>
     </row>
     <row r="12" spans="1:6">
-      <c r="A12" s="98">
+      <c r="A12" s="86">
         <v>621</v>
       </c>
-      <c r="B12" s="98" t="s">
+      <c r="B12" s="86" t="s">
         <v>186</v>
       </c>
-      <c r="C12" s="98" t="s">
+      <c r="C12" s="86" t="s">
         <v>129</v>
       </c>
-      <c r="D12" s="98"/>
-      <c r="E12" s="98"/>
-      <c r="F12" s="98" t="s">
+      <c r="D12" s="86"/>
+      <c r="E12" s="86"/>
+      <c r="F12" s="86" t="s">
         <v>187</v>
       </c>
     </row>
     <row r="13" spans="1:6">
-      <c r="A13" s="98">
+      <c r="A13" s="86">
         <v>624</v>
       </c>
-      <c r="B13" s="98" t="s">
+      <c r="B13" s="86" t="s">
         <v>188</v>
       </c>
-      <c r="C13" s="98" t="s">
+      <c r="C13" s="86" t="s">
         <v>109</v>
       </c>
-      <c r="D13" s="98"/>
-      <c r="E13" s="98"/>
-      <c r="F13" s="98" t="s">
+      <c r="D13" s="86"/>
+      <c r="E13" s="86"/>
+      <c r="F13" s="86" t="s">
         <v>189</v>
       </c>
     </row>
     <row r="14" spans="1:6">
-      <c r="A14" s="98">
+      <c r="A14" s="86">
         <v>625</v>
       </c>
-      <c r="B14" s="98" t="s">
+      <c r="B14" s="86" t="s">
         <v>190</v>
       </c>
-      <c r="C14" s="98" t="s">
+      <c r="C14" s="86" t="s">
         <v>174</v>
       </c>
-      <c r="D14" s="98"/>
-      <c r="E14" s="98"/>
-      <c r="F14" s="98" t="s">
+      <c r="D14" s="86"/>
+      <c r="E14" s="86"/>
+      <c r="F14" s="86" t="s">
         <v>191</v>
       </c>
     </row>
@@ -6416,66 +6407,76 @@
       </c>
     </row>
     <row r="18" ht="18.75" spans="1:6">
-      <c r="A18" s="94">
+      <c r="A18" s="92">
         <v>717</v>
       </c>
-      <c r="B18" s="94" t="s">
+      <c r="B18" s="92" t="s">
         <v>231</v>
       </c>
-      <c r="C18" s="94" t="s">
+      <c r="C18" s="92" t="s">
         <v>109</v>
       </c>
-      <c r="D18" s="94"/>
-      <c r="E18" s="95">
+      <c r="D18" s="92"/>
+      <c r="E18" s="93">
         <v>1830</v>
       </c>
-      <c r="F18" s="95" t="s">
+      <c r="F18" s="93" t="s">
         <v>232</v>
       </c>
     </row>
     <row r="19" ht="18.75" spans="1:6">
-      <c r="A19" s="94">
+      <c r="A19" s="92">
         <v>718</v>
       </c>
-      <c r="B19" s="94" t="s">
+      <c r="B19" s="92" t="s">
         <v>233</v>
       </c>
-      <c r="C19" s="94" t="s">
+      <c r="C19" s="92" t="s">
         <v>109</v>
       </c>
-      <c r="D19" s="94"/>
-      <c r="E19" s="95">
+      <c r="D19" s="92"/>
+      <c r="E19" s="93">
         <v>1831</v>
       </c>
-      <c r="F19" s="94" t="s">
+      <c r="F19" s="92" t="s">
         <v>234</v>
       </c>
     </row>
     <row r="20" ht="18.75" spans="1:6">
-      <c r="A20" s="94">
+      <c r="A20" s="92">
         <v>719</v>
       </c>
-      <c r="B20" s="94" t="s">
+      <c r="B20" s="92" t="s">
         <v>235</v>
       </c>
-      <c r="C20" s="94" t="s">
+      <c r="C20" s="92" t="s">
         <v>167</v>
       </c>
-      <c r="D20" s="94" t="s">
+      <c r="D20" s="92" t="s">
         <v>129</v>
       </c>
-      <c r="E20" s="95"/>
-      <c r="F20" s="95" t="s">
+      <c r="E20" s="93"/>
+      <c r="F20" s="93" t="s">
         <v>236</v>
       </c>
     </row>
-    <row r="21" spans="1:6">
-      <c r="A21" s="96"/>
-      <c r="B21" s="96"/>
-      <c r="C21" s="96"/>
-      <c r="D21" s="96"/>
-      <c r="E21" s="96"/>
-      <c r="F21" s="96"/>
+    <row r="21" ht="37.5" spans="1:6">
+      <c r="A21" s="92">
+        <v>720</v>
+      </c>
+      <c r="B21" s="92" t="s">
+        <v>237</v>
+      </c>
+      <c r="C21" s="92" t="s">
+        <v>129</v>
+      </c>
+      <c r="D21" s="92"/>
+      <c r="E21" s="93" t="s">
+        <v>238</v>
+      </c>
+      <c r="F21" s="93" t="s">
+        <v>239</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -6500,27 +6501,27 @@
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" s="89" t="s">
-        <v>237</v>
+        <v>240</v>
       </c>
       <c r="B1" s="89" t="s">
-        <v>238</v>
+        <v>241</v>
       </c>
       <c r="C1" s="89" t="s">
-        <v>239</v>
+        <v>242</v>
       </c>
       <c r="D1" s="89" t="s">
-        <v>240</v>
+        <v>243</v>
       </c>
       <c r="E1" s="89" t="s">
-        <v>241</v>
+        <v>244</v>
       </c>
     </row>
     <row r="2" s="81" customFormat="1" spans="1:5">
       <c r="A2" s="86" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
       <c r="B2" s="86" t="s">
-        <v>243</v>
+        <v>246</v>
       </c>
       <c r="C2" s="90" t="s">
         <v>150</v>
@@ -6529,15 +6530,15 @@
         <v>129</v>
       </c>
       <c r="E2" s="90" t="s">
-        <v>244</v>
+        <v>247</v>
       </c>
     </row>
     <row r="3" s="81" customFormat="1" spans="1:5">
       <c r="A3" s="86" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
       <c r="B3" s="86" t="s">
-        <v>246</v>
+        <v>249</v>
       </c>
       <c r="C3" s="90" t="s">
         <v>136</v>
@@ -6546,7 +6547,7 @@
         <v>129</v>
       </c>
       <c r="E3" s="90" t="s">
-        <v>247</v>
+        <v>250</v>
       </c>
     </row>
     <row r="4" s="81" customFormat="1" spans="1:5">
@@ -6556,7 +6557,7 @@
         <v>138</v>
       </c>
       <c r="D4" s="90" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="E4" s="90" t="s">
         <v>139</v>
@@ -6588,13 +6589,13 @@
   <sheetData>
     <row r="1" s="81" customFormat="1" spans="1:3">
       <c r="A1" s="88" t="s">
-        <v>249</v>
+        <v>252</v>
       </c>
       <c r="B1" s="88" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
       <c r="C1" s="88" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="2" s="81" customFormat="1" spans="1:3">
@@ -6692,16 +6693,16 @@
   <sheetData>
     <row r="1" s="81" customFormat="1" spans="1:5">
       <c r="A1" s="82" t="s">
-        <v>252</v>
+        <v>255</v>
       </c>
       <c r="B1" s="82" t="s">
-        <v>253</v>
+        <v>256</v>
       </c>
       <c r="C1" s="82" t="s">
-        <v>254</v>
+        <v>257</v>
       </c>
       <c r="D1" s="82" t="s">
-        <v>255</v>
+        <v>258</v>
       </c>
       <c r="E1" s="82" t="s">
         <v>2</v>
@@ -6709,211 +6710,211 @@
     </row>
     <row r="2" s="81" customFormat="1" spans="1:5">
       <c r="A2" s="83" t="s">
-        <v>256</v>
+        <v>259</v>
       </c>
       <c r="B2" s="84" t="s">
-        <v>257</v>
+        <v>260</v>
       </c>
       <c r="C2" s="84">
         <v>1</v>
       </c>
       <c r="D2" s="84" t="s">
-        <v>258</v>
+        <v>261</v>
       </c>
       <c r="E2" s="84" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
     </row>
     <row r="3" s="81" customFormat="1" spans="1:5">
       <c r="A3" s="85" t="s">
-        <v>260</v>
+        <v>263</v>
       </c>
       <c r="B3" s="85" t="s">
-        <v>261</v>
+        <v>264</v>
       </c>
       <c r="C3" s="86">
         <v>1</v>
       </c>
       <c r="D3" s="86" t="s">
-        <v>262</v>
+        <v>265</v>
       </c>
       <c r="E3" s="86" t="s">
-        <v>263</v>
+        <v>266</v>
       </c>
     </row>
     <row r="4" s="81" customFormat="1" spans="1:5">
       <c r="A4" s="85" t="s">
-        <v>264</v>
+        <v>267</v>
       </c>
       <c r="B4" s="86" t="s">
-        <v>265</v>
+        <v>268</v>
       </c>
       <c r="C4" s="86">
         <v>2</v>
       </c>
       <c r="D4" s="86" t="s">
-        <v>262</v>
+        <v>265</v>
       </c>
       <c r="E4" s="86" t="s">
-        <v>266</v>
+        <v>269</v>
       </c>
     </row>
     <row r="5" s="81" customFormat="1" spans="1:5">
       <c r="A5" s="85" t="s">
-        <v>267</v>
+        <v>270</v>
       </c>
       <c r="B5" s="86" t="s">
-        <v>268</v>
+        <v>271</v>
       </c>
       <c r="C5" s="86">
         <v>20</v>
       </c>
       <c r="D5" s="86" t="s">
-        <v>262</v>
+        <v>265</v>
       </c>
       <c r="E5" s="86" t="s">
-        <v>269</v>
+        <v>272</v>
       </c>
     </row>
     <row r="6" s="81" customFormat="1" spans="1:5">
       <c r="A6" s="83" t="s">
-        <v>270</v>
+        <v>273</v>
       </c>
       <c r="B6" s="84" t="s">
-        <v>265</v>
+        <v>268</v>
       </c>
       <c r="C6" s="84">
         <v>1</v>
       </c>
       <c r="D6" s="84" t="s">
-        <v>258</v>
+        <v>261</v>
       </c>
       <c r="E6" s="84" t="s">
-        <v>271</v>
+        <v>274</v>
       </c>
     </row>
     <row r="7" s="81" customFormat="1" spans="1:5">
       <c r="A7" s="83" t="s">
-        <v>272</v>
+        <v>275</v>
       </c>
       <c r="B7" s="84" t="s">
-        <v>268</v>
+        <v>271</v>
       </c>
       <c r="C7" s="84">
         <v>80</v>
       </c>
       <c r="D7" s="84" t="s">
-        <v>258</v>
+        <v>261</v>
       </c>
       <c r="E7" s="84" t="s">
-        <v>273</v>
+        <v>276</v>
       </c>
     </row>
     <row r="8" s="81" customFormat="1" spans="1:5">
       <c r="A8" s="83" t="s">
-        <v>274</v>
+        <v>277</v>
       </c>
       <c r="B8" s="84" t="s">
-        <v>268</v>
+        <v>271</v>
       </c>
       <c r="C8" s="84">
         <v>80</v>
       </c>
       <c r="D8" s="84" t="s">
-        <v>258</v>
+        <v>261</v>
       </c>
       <c r="E8" s="84" t="s">
-        <v>247</v>
+        <v>250</v>
       </c>
     </row>
     <row r="9" s="81" customFormat="1" spans="1:5">
       <c r="A9" s="83" t="s">
-        <v>275</v>
+        <v>278</v>
       </c>
       <c r="B9" s="84" t="s">
-        <v>276</v>
+        <v>279</v>
       </c>
       <c r="C9" s="84">
         <v>4</v>
       </c>
       <c r="D9" s="84" t="s">
-        <v>258</v>
+        <v>261</v>
       </c>
       <c r="E9" s="84" t="s">
-        <v>277</v>
+        <v>280</v>
       </c>
     </row>
     <row r="10" s="81" customFormat="1" spans="1:5">
       <c r="A10" s="83" t="s">
-        <v>278</v>
+        <v>281</v>
       </c>
       <c r="B10" s="86" t="s">
-        <v>265</v>
+        <v>268</v>
       </c>
       <c r="C10" s="86">
         <v>2</v>
       </c>
       <c r="D10" s="86" t="s">
-        <v>262</v>
+        <v>265</v>
       </c>
       <c r="E10" s="86" t="s">
-        <v>279</v>
+        <v>282</v>
       </c>
     </row>
     <row r="11" s="81" customFormat="1" spans="1:5">
       <c r="A11" s="83" t="s">
-        <v>280</v>
+        <v>283</v>
       </c>
       <c r="B11" s="84" t="s">
-        <v>265</v>
+        <v>268</v>
       </c>
       <c r="C11" s="84">
         <v>2</v>
       </c>
       <c r="D11" s="84" t="s">
-        <v>258</v>
+        <v>261</v>
       </c>
       <c r="E11" s="84" t="s">
-        <v>281</v>
+        <v>284</v>
       </c>
     </row>
     <row r="12" s="81" customFormat="1" spans="1:5">
       <c r="A12" s="83" t="s">
-        <v>280</v>
+        <v>283</v>
       </c>
       <c r="B12" s="84" t="s">
-        <v>268</v>
+        <v>271</v>
       </c>
       <c r="C12" s="84">
         <v>80</v>
       </c>
       <c r="D12" s="84" t="s">
-        <v>258</v>
+        <v>261</v>
       </c>
       <c r="E12" s="84" t="s">
-        <v>282</v>
+        <v>285</v>
       </c>
     </row>
     <row r="13" s="81" customFormat="1" spans="1:5">
       <c r="A13" s="83" t="s">
-        <v>280</v>
+        <v>283</v>
       </c>
       <c r="B13" s="84" t="s">
-        <v>265</v>
+        <v>268</v>
       </c>
       <c r="C13" s="84">
         <v>2</v>
       </c>
       <c r="D13" s="84" t="s">
-        <v>258</v>
+        <v>261</v>
       </c>
       <c r="E13" s="84" t="s">
-        <v>283</v>
+        <v>286</v>
       </c>
     </row>
     <row r="14" s="81" customFormat="1" spans="1:5">
       <c r="A14" s="87" t="s">
-        <v>284</v>
+        <v>287</v>
       </c>
       <c r="B14" s="86"/>
       <c r="C14" s="86"/>
@@ -6922,70 +6923,70 @@
     </row>
     <row r="15" s="81" customFormat="1" spans="1:5">
       <c r="A15" s="85" t="s">
-        <v>285</v>
+        <v>288</v>
       </c>
       <c r="B15" s="86" t="s">
-        <v>265</v>
+        <v>268</v>
       </c>
       <c r="C15" s="86">
         <v>2</v>
       </c>
       <c r="D15" s="86" t="s">
-        <v>262</v>
+        <v>265</v>
       </c>
       <c r="E15" s="86" t="s">
-        <v>286</v>
+        <v>289</v>
       </c>
     </row>
     <row r="16" s="81" customFormat="1" spans="1:5">
       <c r="A16" s="85" t="s">
-        <v>287</v>
+        <v>290</v>
       </c>
       <c r="B16" s="86" t="s">
-        <v>268</v>
+        <v>271</v>
       </c>
       <c r="C16" s="86">
         <v>80</v>
       </c>
       <c r="D16" s="86" t="s">
-        <v>262</v>
+        <v>265</v>
       </c>
       <c r="E16" s="86" t="s">
-        <v>288</v>
+        <v>291</v>
       </c>
     </row>
     <row r="17" s="81" customFormat="1" ht="12" customHeight="1" spans="1:5">
       <c r="A17" s="83" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="B17" s="84" t="s">
-        <v>265</v>
+        <v>268</v>
       </c>
       <c r="C17" s="84">
         <v>2</v>
       </c>
       <c r="D17" s="84" t="s">
-        <v>258</v>
+        <v>261</v>
       </c>
       <c r="E17" s="84" t="s">
-        <v>290</v>
+        <v>293</v>
       </c>
     </row>
     <row r="18" s="81" customFormat="1" spans="1:5">
       <c r="A18" s="85" t="s">
-        <v>285</v>
+        <v>288</v>
       </c>
       <c r="B18" s="84" t="s">
-        <v>265</v>
+        <v>268</v>
       </c>
       <c r="C18" s="84">
         <v>2</v>
       </c>
       <c r="D18" s="84" t="s">
-        <v>258</v>
+        <v>261</v>
       </c>
       <c r="E18" s="84" t="s">
-        <v>291</v>
+        <v>294</v>
       </c>
     </row>
   </sheetData>
@@ -7009,13 +7010,13 @@
   <sheetData>
     <row r="1" ht="16.5" spans="1:4">
       <c r="A1" s="5" t="s">
-        <v>292</v>
+        <v>295</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>293</v>
+        <v>296</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>294</v>
+        <v>297</v>
       </c>
     </row>
     <row r="2" ht="16.5" spans="1:4">
@@ -7023,10 +7024,10 @@
         <v>0</v>
       </c>
       <c r="B2" s="78" t="s">
-        <v>295</v>
+        <v>298</v>
       </c>
       <c r="C2" s="26" t="s">
-        <v>296</v>
+        <v>299</v>
       </c>
     </row>
     <row r="3" ht="16.5" spans="1:4">
@@ -7034,13 +7035,13 @@
         <v>1</v>
       </c>
       <c r="B3" s="78" t="s">
-        <v>297</v>
+        <v>300</v>
       </c>
       <c r="C3" s="79" t="s">
-        <v>296</v>
+        <v>299</v>
       </c>
       <c r="D3" s="80" t="s">
-        <v>298</v>
+        <v>301</v>
       </c>
     </row>
     <row r="4" ht="16.5" spans="1:4">
@@ -7048,10 +7049,10 @@
         <v>10</v>
       </c>
       <c r="B4" s="78" t="s">
-        <v>299</v>
+        <v>302</v>
       </c>
       <c r="C4" s="26" t="s">
-        <v>300</v>
+        <v>303</v>
       </c>
       <c r="D4" s="80"/>
     </row>
@@ -7060,10 +7061,10 @@
         <v>100</v>
       </c>
       <c r="B5" s="24" t="s">
-        <v>301</v>
+        <v>304</v>
       </c>
       <c r="C5" s="26" t="s">
-        <v>300</v>
+        <v>303</v>
       </c>
       <c r="D5" s="80"/>
     </row>
@@ -7072,10 +7073,10 @@
         <v>200</v>
       </c>
       <c r="B6" s="24" t="s">
-        <v>302</v>
+        <v>305</v>
       </c>
       <c r="C6" s="26" t="s">
-        <v>300</v>
+        <v>303</v>
       </c>
       <c r="D6" s="80"/>
     </row>

</xml_diff>